<commit_message>
Refactored framework and added API automation support
</commit_message>
<xml_diff>
--- a/TestData/data.xlsx
+++ b/TestData/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Java Student\Hybrid_Framework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{936A3B23-DAA1-44A0-BA15-63B34E95E71E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5084871E-C0F0-49C1-808A-28B12C37F000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="57">
   <si>
     <t>Vishal@gmail.com</t>
   </si>
@@ -196,6 +196,9 @@
   </si>
   <si>
     <t>Vishal3@gamail.com</t>
+  </si>
+  <si>
+    <t>Seleium</t>
   </si>
 </sst>
 </file>
@@ -544,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -576,6 +579,11 @@
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>